<commit_message>
Mise à jour cardinalités (#263)
* update cardinalities

* fix

* ordering ac8b7c95df57bb64237458f12c9f332bb4fd0f72
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-as-dp-device.xlsx
+++ b/main/ig/StructureDefinition-as-dp-device.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-03-18T16:59:29+00:00</t>
+    <t>2025-03-21T10:50:44+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -7723,7 +7723,7 @@
       </c>
       <c r="E50" s="2"/>
       <c r="F50" t="s" s="2">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="G50" t="s" s="2">
         <v>79</v>
@@ -7839,7 +7839,7 @@
       </c>
       <c r="E51" s="2"/>
       <c r="F51" t="s" s="2">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="G51" t="s" s="2">
         <v>86</v>

</xml_diff>